<commit_message>
Use template color values in writing guide and checklist
Palette now matches the proposal templates: Dark Purple 51389D, Lilac
F2EFFE, Light Grey EFF4FC, Dark Grey 888888. Guide heading styles, title
block and tables rebuilt to its own typography and table rules; section
numbering made sequential; Vibrant Purple renamed Bright Purple.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014SmHRydJLVa8K2jN5veRpq
</commit_message>
<xml_diff>
--- a/skills/proposal-structure-generator/assets/checklist_public_partners.xlsx
+++ b/skills/proposal-structure-generator/assets/checklist_public_partners.xlsx
@@ -31,13 +31,13 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="0052389D"/>
+      <color rgb="0051389D"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00919191"/>
+      <color rgb="00888888"/>
       <sz val="10"/>
     </font>
     <font>
@@ -66,7 +66,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="0052389D"/>
+      <color rgb="0051389D"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -79,12 +79,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0052389D"/>
+        <fgColor rgb="0051389D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1EFFD"/>
+        <fgColor rgb="00F2EFFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,7 +98,7 @@
     </border>
     <border>
       <bottom style="thin">
-        <color rgb="00F1EFFD"/>
+        <color rgb="00F2EFFE"/>
       </bottom>
     </border>
   </borders>
@@ -161,12 +161,12 @@
     <dxf>
       <font>
         <b val="1"/>
-        <color rgb="0052389D"/>
+        <color rgb="0051389D"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <color rgb="00919191"/>
+        <color rgb="00888888"/>
       </font>
     </dxf>
   </dxfs>

</xml_diff>